<commit_message>
Fix all errors: Markdown parsing, note capture, reroute preservation, and robust excel export
</commit_message>
<xml_diff>
--- a/Маршрут_Астана_готовый.xlsx
+++ b/Маршрут_Астана_готовый.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Маршрут" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ссылки Google Maps" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Не найдены" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Маршрут" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ссылки Google Maps" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Не найдены" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,34 +577,34 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Express market GS</t>
+          <t>667 алкомаркет GS</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>ул. Туран 55/1</t>
+          <t>ул. Анет баба 2</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Калилаев</t>
+          <t>Манас Жамал Бауыржановна</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Турехан Калилаев</t>
+          <t>Жамал Манас</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>+7 747 190 1010</t>
+          <t>+7 702 222 0723</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -628,34 +628,34 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Tau.ortalygy GS</t>
+          <t>Хозяйн GS</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ул. Бухар Жырау 34/2</t>
+          <t>ул. Мухамедханов 21/2, ВП 6</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Акмарал</t>
+          <t>Тайбагарова М.М.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Акмарал</t>
+          <t>Мира Тайбагарова</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>+7 701 510 3030</t>
+          <t>+7 777 644 1441</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -679,34 +679,34 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Дармакс GS</t>
+          <t>Базар маркет GS</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>ул. Е 652, 22, ЖК AruPark-3</t>
+          <t>ул. Азильхана Нуршайыкова 10/1</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Салкимбаева</t>
+          <t>Айзат</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Азамат Салкимбаев</t>
+          <t>Айзат Тукибаева</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>+7 705 613 4270</t>
+          <t>+7 775 492 8077</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -730,34 +730,34 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Arumarket GS</t>
+          <t>Express market GS</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ул. Е 652, 22, ЖК AruPark-3</t>
+          <t>ул. Туран 55/1</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Салкимбаева</t>
+          <t>Калилаев</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Азамат Салкимбаев</t>
+          <t>Турехан Калилаев</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>+7 705 613 4270</t>
+          <t>+7 747 190 1010</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -781,34 +781,34 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Бестобе GS</t>
+          <t>Tau.ortalygy GS</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ул. Туркестан 30, НП 3</t>
+          <t>ул. Бухар Жырау 34/2</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Баймуханов</t>
+          <t>Акмарал</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Адилет Баймуханов</t>
+          <t>Акмарал</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>+7 705 669 6131</t>
+          <t>+7 701 510 3030</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -832,34 +832,34 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Bope Star GS</t>
+          <t>Arumarket GS</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ул. Акмешит 1/1</t>
+          <t>ул. Е 652, 22, ЖК AruPark-3</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Gelsomino</t>
+          <t>Салкимбаева</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Ди</t>
+          <t>Азамат Салкимбаев</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>+7 701 088 0908</t>
+          <t>+7 705 613 4270</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -883,34 +883,34 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Сәтті GS</t>
+          <t>Дармакс GS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>ул. Шакарим Кудайберди 25/1</t>
+          <t>ул. Е 652, 22, ЖК AruPark-3</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Омар</t>
+          <t>Салкимбаева</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Гаухар Омар</t>
+          <t>Азамат Салкимбаев</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>+7 707 503 9797</t>
+          <t>+7 705 613 4270</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -934,34 +934,34 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Aqmol GS</t>
+          <t>Бестобе GS</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ул. Сарайшык 5/4</t>
+          <t>ул. Туркестан 30, НП 3</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Soft Line</t>
+          <t>Баймуханов</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Айжан Уразбаева</t>
+          <t>Адилет Баймуханов</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>+7 705 498 1111</t>
+          <t>+7 705 669 6131</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -985,34 +985,34 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Султан GS</t>
+          <t>Bope Star GS</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ул. Аль-Фараби 35, 14</t>
+          <t>ул. Акмешит 1/1</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Нуркасымова</t>
+          <t>Gelsomino</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Гульсум Нуркасымова</t>
+          <t>Ди</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>+7 705 888 0803</t>
+          <t>+7 701 088 0908</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
@@ -1036,34 +1036,34 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>NUR-KB GS</t>
+          <t>Сәтті GS</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Алматинский район, ул. 23-16, дом 39</t>
+          <t>ул. Шакарим Кудайберди 25/1</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>ТОО Нур-КБ</t>
+          <t>Омар</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Искендер Оторбаев</t>
+          <t>Гаухар Омар</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>+7 708 946 0803</t>
+          <t>+7 707 503 9797</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -1087,34 +1087,34 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>AVO MARKET GS</t>
+          <t>Aqmol GS</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ул. Момышулы 2в</t>
+          <t>ул. Сарайшык 5/4</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Иманмагзамова</t>
+          <t>Soft Line</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Гульнар Иманмагзамова</t>
+          <t>Айжан Уразбаева</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>+7 771 163 3625</t>
+          <t>+7 705 498 1111</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -1138,34 +1138,34 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Байлык GS</t>
+          <t>AVO MARKET GS</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ул. А 52, 2</t>
+          <t>ул. Момышулы 2в</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Токешова С.А.</t>
+          <t>Иманмагзамова</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Светлана Токешова</t>
+          <t>Гульнар Иманмагзамова</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>+7 747 676 8819</t>
+          <t>+7 771 163 3625</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
@@ -1189,34 +1189,34 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Ғажап GS</t>
+          <t>Байлык GS</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>ул. А 52, дом 4</t>
+          <t>ул. А 52, 2</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Айткельдиев Азамат Жанатович</t>
+          <t>Токешова С.А.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Азамат Айткельдиев</t>
+          <t>Светлана Токешова</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>+7 778 764 5558</t>
+          <t>+7 747 676 8819</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
@@ -1240,34 +1240,34 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Ернұр GS</t>
+          <t>Ғажап GS</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>ул. А. Байтұрсынов 22</t>
+          <t>ул. А 52, дом 4</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Ер-Нур</t>
+          <t>Айткельдиев Азамат Жанатович</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ер-Нұр</t>
+          <t>Азамат Айткельдиев</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>+7 705 376 0494</t>
+          <t>+7 778 764 5558</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
@@ -1291,30 +1291,34 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Saturn GS</t>
+          <t>Ернұр GS</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>ул. Байтурсынова 39/2, ЖК Сатурн</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
+          <t>ул. А. Байтұрсынов 22</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Ер-Нур</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Гульжанат</t>
+          <t>Ер-Нұр</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>+7 747 975 9696</t>
+          <t>+7 705 376 0494</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1338,34 +1342,30 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Нур GS</t>
+          <t>Saturn GS</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ул. Кордай 36/1</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Оспанов А.</t>
-        </is>
-      </c>
+          <t>ул. Байтурсынова 39/2, ЖК Сатурн</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Арман Оспанов</t>
+          <t>Гульжанат</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>+7 701 203 8662</t>
+          <t>+7 747 975 9696</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -1389,34 +1389,34 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Военторг GS</t>
+          <t>Нур GS</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>ул. Абылай хана 29/1</t>
+          <t>ул. Кордай 36/1</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Косуакова Айсамал Самбетовна</t>
+          <t>Оспанов А.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Айсамал Косуакова</t>
+          <t>Арман Оспанов</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>+7 775 933 6666</t>
+          <t>+7 701 203 8662</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
@@ -1440,31 +1440,31 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Магазин Сигарет GS</t>
+          <t>Военторг GS</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Шоссе Алаш 31/1, рынок Шарын</t>
+          <t>ул. Абылай хана 29/1</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>ИП Маханбетияр</t>
+          <t>Косуакова Айсамал Самбетовна</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Дана Маханбетияр</t>
+          <t>Айсамал Косуакова</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>+7 702 908 9202</t>
+          <t>+7 775 933 6666</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>82</v>
@@ -1491,38 +1491,38 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Danial GS</t>
+          <t>NUR-KB GS</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>пр. Абая 48, ТД Жаннур, бутик А6</t>
+          <t>Алматинский район, ул. 23-16, дом 39</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Даниал</t>
+          <t>ТОО Нур-КБ</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Галина Мамбетова</t>
+          <t>Искендер Оторбаев</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>+7 702 448 8886</t>
+          <t>+7 708 946 0803</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>кэш</t>
+          <t>OSM</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -1542,34 +1542,34 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Хозяйн GS</t>
+          <t>Danial GS</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>ул. Мухамедханов 21/2, ВП 6</t>
+          <t>пр. Абая 48, ТД Жаннур, бутик А6</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Тайбагарова М.М.</t>
+          <t>Даниал</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Мира Тайбагарова</t>
+          <t>Галина Мамбетова</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>+7 777 644 1441</t>
+          <t>+7 702 448 8886</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
@@ -1593,38 +1593,38 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>667 алкомаркет GS</t>
+          <t>Султан GS</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>ул. Анет баба 2</t>
+          <t>ул. Аль-Фараби 35, 14</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Манас Жамал Бауыржановна</t>
+          <t>Нуркасымова</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Жамал Манас</t>
+          <t>Гульсум Нуркасымова</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>+7 702 222 0723</t>
+          <t>+7 705 888 0803</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>кэш</t>
+          <t>OSM</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -1644,34 +1644,34 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Базар маркет GS</t>
+          <t>Магазин Сигарет GS</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>ул. Азильхана Нуршайыкова 10/1</t>
+          <t>Шоссе Алаш 31/1, рынок Шарын</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Айзат</t>
+          <t>ИП Маханбетияр</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Айзат Тукибаева</t>
+          <t>Дана Маханбетияр</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>+7 775 492 8077</t>
+          <t>+7 702 908 9202</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -1719,10 +1719,10 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
         <v>15</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -1794,7 +1794,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Время в пути по дорогам без учёта пробок и стоянок: около 132 мин.</t>
+          <t>Время в пути по дорогам без учёта пробок и стоянок: около 130 мин.</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Султан GS</t>
+          <t>Bope Star GS</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1927,12 +1927,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Султан GS</t>
+          <t>Bope Star GS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Магазин Сигарет GS</t>
+          <t>Военторг GS</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Магазин Сигарет GS</t>
+          <t>Военторг GS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>